<commit_message>
Put the pack count back in the cell, not in a footnote
I left the per-set Packs cells blank on the two multi-set rows and moved the
logged total into Notes, on the reasoning that 18 across five sets does not
say how many came from each and the sheet should not invent a split.

The reasoning holds and the decision was still wrong. It left Tim looking at
empty cells where he had typed a number, which reads as data loss whatever a
note says, and he had already told me the number twice. He knows the split
and can move a figure across four columns in seconds; what he cannot do is
recover a number the sheet decided not to show him.

The total now lands in the first set's cell, so Packs Opened sums to 18 and 6
straight away, and the note says to spread it if the packs came from
different sets. Single-set rows are untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Garbage-Rips-585-Video-Log.xlsx
+++ b/Garbage-Rips-585-Video-Log.xlsx
@@ -26256,7 +26256,9 @@
           <t>Phantasmal Flames</t>
         </is>
       </c>
-      <c r="H311" s="14" t="n"/>
+      <c r="H311" s="15" t="n">
+        <v>18</v>
+      </c>
       <c r="I311" s="14" t="inlineStr">
         <is>
           <t>Destined Rivals</t>
@@ -26320,7 +26322,7 @@
       <c r="AD311" s="15" t="n"/>
       <c r="AE311" s="15" t="inlineStr">
         <is>
-          <t>Previously logged 18 packs in total. Split it across the Packs columns.</t>
+          <t>All 18 packs are on the first set. Move some across the Packs columns if they came from different sets.</t>
         </is>
       </c>
     </row>
@@ -26357,7 +26359,9 @@
           <t>Mega Evolution</t>
         </is>
       </c>
-      <c r="H312" s="15" t="n"/>
+      <c r="H312" s="15" t="n">
+        <v>6</v>
+      </c>
       <c r="I312" s="14" t="inlineStr">
         <is>
           <t>Destined Rivals</t>
@@ -26421,7 +26425,7 @@
       <c r="AD312" s="15" t="n"/>
       <c r="AE312" s="15" t="inlineStr">
         <is>
-          <t>Previously logged 6 packs in total. Split it across the Packs columns.</t>
+          <t>All 6 packs are on the first set. Move some across the Packs columns if they came from different sets.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Give the video log a filter, which is the fix that actually changes the work
The log is sorted newest first, which is right for "I just uploaded, log it".
Tim backfills the other way, oldest first, and there was no autofilter, so that
meant scrolling to row 314 every session and finding the next blank by eye.

With a filter he sorts Published ascending in one click and can filter any
column to Blanks to see exactly what is left. It survives into Google Sheets as
the standard filter.

The Summary tab also never counted the rarity column, which is the one with the
most left to do, so the progress readout looked further along than the work
was. Rarity and pack counts are counted now, with a remaining figure for packs.

Re-verified after the rebuild: 661 filled cells across every validated column
and zero failing validation, all seven list ranges matching their contents
exactly, 313 rows, six header notes, panes frozen.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Garbage-Rips-585-Video-Log.xlsx
+++ b/Garbage-Rips-585-Video-Log.xlsx
@@ -16,7 +16,9 @@
     <sheet name="My Hits" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Shops" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Video Log'!$A$1:$AE$314</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -26768,6 +26770,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AE314"/>
   <dataValidations count="14">
     <dataValidation sqref="G2:G314" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Lists!$A$2:$A$39</formula1>
@@ -27499,7 +27502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -27571,82 +27574,115 @@
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Opening type filled in</t>
+          <t>Hit rarity filled in</t>
         </is>
       </c>
       <c r="B8" s="18">
-        <f>COUNTA('Video Log'!R2:R314)</f>
+        <f>COUNTA('Video Log'!V2:V314)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Marked as a hit</t>
+          <t>Pack count filled in</t>
         </is>
       </c>
       <c r="B9" s="18">
-        <f>COUNTIF('Video Log'!T2:T314,"Yes")</f>
+        <f>COUNTA('Video Log'!H2:H314)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Hit card named</t>
+          <t>Still missing a pack count</t>
         </is>
       </c>
       <c r="B10" s="18">
-        <f>COUNTA('Video Log'!U2:U314)</f>
+        <f>COUNTA('Video Log'!A2:A314)-COUNTA('Video Log'!H2:H314)</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>In Greatest Hits</t>
+          <t>Opening type filled in</t>
         </is>
       </c>
       <c r="B11" s="18">
-        <f>COUNTIF('Video Log'!W2:W314,"Yes")</f>
+        <f>COUNTA('Video Log'!R2:R314)</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Given a rank</t>
+          <t>Marked as a hit</t>
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTA('Video Log'!X2:X314)</f>
+        <f>COUNTIF('Video Log'!T2:T314,"Yes")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>Affiliate links added</t>
+          <t>Hit card named</t>
         </is>
       </c>
       <c r="B13" s="18">
-        <f>COUNTA('Video Log'!Z2:Z314)</f>
+        <f>COUNTA('Video Log'!U2:U314)</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
+          <t>In Greatest Hits</t>
+        </is>
+      </c>
+      <c r="B14" s="18">
+        <f>COUNTIF('Video Log'!W2:W314,"Yes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Given a rank</t>
+        </is>
+      </c>
+      <c r="B15" s="18">
+        <f>COUNTA('Video Log'!X2:X314)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Affiliate links added</t>
+        </is>
+      </c>
+      <c r="B16" s="18">
+        <f>COUNTA('Video Log'!Z2:Z314)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
           <t>Hidden from the site</t>
         </is>
       </c>
-      <c r="B14" s="18">
+      <c r="B17" s="18">
         <f>COUNTIF('Video Log'!AD2:AD314,"Yes")</f>
         <v/>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Counts update as you type. Blank cells are skipped by the import, so a half-filled sheet is fine.</t>
         </is>

</xml_diff>

<commit_message>
Today's rip: Ascended Heroes single pack #9, no hit
zrI6oaxBct8, 30 August 2026. Single Booster Pack, pack 9, no hit,
Ascended Heroes. Row 329 of the Video Log, all ten Summary ranges
extended, imported and synced in the documented order: import-sheet.mjs
first so manual.json exists, then sync-youtube.mjs to merge it.

AND THE SHOW HANDOVER COMPLETED ITS FIRST FULL CYCLE, which is the thing
the owner asked to watch. Yesterday GI Cards was on the calendar and
hidden on the archive; today it is off the calendar and VISIBLE on the
archive, and CollectorFest has taken its place as today's show, present
on the archive but hidden until tomorrow. The rule he asked for -- a show
stays on the calendar through its own day and moves the day after -- now
has two days of evidence rather than an argument.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Garbage-Rips-585-Video-Log.xlsx
+++ b/Garbage-Rips-585-Video-Log.xlsx
@@ -6436,7 +6436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U328"/>
+  <dimension ref="A1:U329"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -27267,6 +27267,53 @@
       <c r="L328" t="inlineStr">
         <is>
           <t>Chaos Rising</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>zrI6oaxBct8</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Ascended Heroes is TOUGH 💀🤘</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="D329" t="n">
+        <v>106</v>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>0:21</t>
+        </is>
+      </c>
+      <c r="F329">
+        <f>HYPERLINK("https://youtu.be/zrI6oaxBct8","watch")</f>
+        <v/>
+      </c>
+      <c r="H329" t="inlineStr">
+        <is>
+          <t>Single Booster Pack</t>
+        </is>
+      </c>
+      <c r="I329" t="n">
+        <v>9</v>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>Ascended Heroes</t>
         </is>
       </c>
     </row>
@@ -28121,7 +28168,7 @@
         </is>
       </c>
       <c r="B3" s="18">
-        <f>COUNTA('Video Log'!A2:A328)</f>
+        <f>COUNTA('Video Log'!A2:A329)</f>
         <v/>
       </c>
     </row>
@@ -28132,7 +28179,7 @@
         </is>
       </c>
       <c r="B4" s="18">
-        <f>COUNTA('Video Log'!H2:H328)</f>
+        <f>COUNTA('Video Log'!H2:H329)</f>
         <v/>
       </c>
     </row>
@@ -28143,7 +28190,7 @@
         </is>
       </c>
       <c r="B5" s="18">
-        <f>COUNTA('Video Log'!A2:A328)-COUNTA('Video Log'!H2:H328)</f>
+        <f>COUNTA('Video Log'!A2:A329)-COUNTA('Video Log'!H2:H329)</f>
         <v/>
       </c>
     </row>
@@ -28154,7 +28201,7 @@
         </is>
       </c>
       <c r="B6" s="18">
-        <f>COUNTA('Video Log'!L2:L328)</f>
+        <f>COUNTA('Video Log'!L2:L329)</f>
         <v/>
       </c>
     </row>
@@ -28165,7 +28212,7 @@
         </is>
       </c>
       <c r="B7" s="18">
-        <f>COUNTA('Video Log'!A2:A328)-COUNTA('Video Log'!L2:L328)</f>
+        <f>COUNTA('Video Log'!A2:A329)-COUNTA('Video Log'!L2:L329)</f>
         <v/>
       </c>
     </row>
@@ -28176,7 +28223,7 @@
         </is>
       </c>
       <c r="B8" s="18">
-        <f>COUNTA('Video Log'!I2:I328)</f>
+        <f>COUNTA('Video Log'!I2:I329)</f>
         <v/>
       </c>
     </row>
@@ -28187,7 +28234,7 @@
         </is>
       </c>
       <c r="B9" s="18">
-        <f>COUNTIF('Video Log'!J2:J328,"Yes")</f>
+        <f>COUNTIF('Video Log'!J2:J329,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -28198,7 +28245,7 @@
         </is>
       </c>
       <c r="B10" s="18">
-        <f>COUNTA('Video Log'!K2:K328)</f>
+        <f>COUNTA('Video Log'!K2:K329)</f>
         <v/>
       </c>
     </row>
@@ -28209,7 +28256,7 @@
         </is>
       </c>
       <c r="B11" s="18">
-        <f>COUNTIF('Video Log'!M2:M328,"Yes")</f>
+        <f>COUNTIF('Video Log'!M2:M329,"Yes")</f>
         <v/>
       </c>
     </row>
@@ -28220,7 +28267,7 @@
         </is>
       </c>
       <c r="B12" s="18">
-        <f>COUNTA('Video Log'!N2:N328)</f>
+        <f>COUNTA('Video Log'!N2:N329)</f>
         <v/>
       </c>
     </row>

</xml_diff>